<commit_message>
Rename ts_ARIMA to ts_HoltWinters and sync latest data files
- model_results.json + train_all_models.py: correct forecast model key
  from ts_ARIMA to ts_HoltWinters (Holt-Winters is what was actually run)
- PargoParcels_Analytics.xlsx: latest workbook build
- dbt_performance_review.csv: add dbt run performance report
</commit_message>
<xml_diff>
--- a/PargoParcels_Analytics.xlsx
+++ b/PargoParcels_Analytics.xlsx
@@ -25,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,8 +84,13 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -122,6 +127,11 @@
         <fgColor rgb="00F59E0B"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -135,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -176,6 +186,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -542,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -569,7 +582,7 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
+    <row r="3" ht="36" customHeight="1"/>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -747,9 +760,18 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>Data note: Workbook figures summarise the enterprise-scale portfolio dataset. Other workbook samples, dashboards, and ebooks may use different scopes; ML metrics use held-out validation data and business impact values are modelled estimates.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
     <mergeCell ref="B14:H14"/>
+    <mergeCell ref="A3:H3"/>
     <mergeCell ref="B9:H9"/>
     <mergeCell ref="B13:H13"/>
     <mergeCell ref="A2:H2"/>
@@ -758,6 +780,7 @@
     <mergeCell ref="B10:H10"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B11:H11"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>